<commit_message>
Fix row order: August entries were sitting after September
The 13 rows appended for the EAO tickets were in ticket-number order, not
date order -- the two GM sub-events (Aug 3) ended up after EAO-33/34
(Sep 2-3). Re-sorted the appended block chronologically in both
customer_tracker.csv and the xlsx Data sheet (direct row-content swap via
XML, not an openpyxl resave, to avoid re-stripping the dynamic-array
metadata fixed earlier). The original 80 rows were already in correct
order and were left untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FHaiZAbQ4hsiftTWXhdhmi
</commit_message>
<xml_diff>
--- a/EventWatch_Customer_Complaints_2026.xlsx
+++ b/EventWatch_Customer_Complaints_2026.xlsx
@@ -12171,16 +12171,16 @@
         <v>46235</v>
       </c>
       <c r="B89" s="119" t="n">
-        <v>46251</v>
+        <v>46237</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Transport Disruption</t>
+          <t>Factory Fire</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Eaton</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="E89" t="n">
@@ -12188,27 +12188,27 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Kandla Port Cargo Congestion – Supplier Impact Notification Clarification (Eaton)</t>
+          <t>Fire at UTAS-Nova Automotive Lighting Systems, Danyang, Jiangsu, China</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Inquiry</t>
+          <t>Complaint</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Supplier Impact Mapping Clarification</t>
+          <t>Missed Event</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Mapping</t>
+          <t>Source Coverage</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -12218,27 +12218,27 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>Clarification Provided</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Impact-confirmation notification criteria documentation for port/logistics bulletins</t>
+          <t>Chinese regional source coverage for sub-tier automotive lighting suppliers</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Staged from Jira EAO-28 (Done). Eaton asked what criteria triggered impact-confirmation notifications to Eaton suppliers on the Kandla Port cargo congestion bulletin, since the bulletin text focused on rice exports.</t>
+          <t>Staged from Jira EAO-25 (Sent to PM). GM reported a fire at UTAS-Nova Automotive Lighting Systems, Danyang, Jiangsu, China (reported July 10) was not found in GM's org; investigation findings not yet shared, Short Term Fix Status set to Pending until CS responds.</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="R89" t="n">
@@ -12249,17 +12249,17 @@
       </c>
       <c r="U89" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="V89" t="inlineStr">
         <is>
-          <t>Entity &amp; Supplier Resolution</t>
+          <t>Dynamic Source Discovery</t>
         </is>
       </c>
       <c r="W89" t="inlineStr">
         <is>
-          <t>EAO-28</t>
+          <t>EAO-25</t>
         </is>
       </c>
     </row>
@@ -12268,16 +12268,16 @@
         <v>46235</v>
       </c>
       <c r="B90" s="119" t="n">
-        <v>46265</v>
+        <v>46237</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Tornado</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Liberty Blume</t>
+          <t>GM</t>
         </is>
       </c>
       <c r="E90" t="n">
@@ -12285,27 +12285,27 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Ciena 400G Optics Counterfeit Risk Intelligence Request (Liberty Blume)</t>
+          <t>Chicago Heights, Illinois Tornado – Trialco Impact Not Identified</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Inquiry</t>
+          <t>Complaint</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Intelligence/Advisory Request</t>
+          <t>Missed Event</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>People</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Process Clarification</t>
+          <t>Event Identification</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -12320,22 +12320,22 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Counterfeit/grey-market component intelligence briefing capability</t>
+          <t>Escalation automation for localized-impact tornado/storm sub-events and named-facility (Trialco) impact confirmation</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>Staged from Jira EAO-32 (Open). Liberty Blume requested industry intelligence on counterfeit/grey-market Ciena 400G optical transceivers beyond the supplier scanning report already provided.</t>
+          <t>Staged from Jira EAO-25 (Sent to PM). GM reported no event was created specifically for the July 27 Chicago Heights, Illinois tornado (broader Illinois storm alerts existed) and asked whether Trialco was identified as impacted; investigation findings not yet shared, Short Term Fix Status set to Pending until CS responds.</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="R90" t="n">
@@ -12346,35 +12346,35 @@
       </c>
       <c r="U90" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="V90" t="inlineStr">
         <is>
-          <t>Other Control Automation</t>
+          <t>WarRoom &amp; Decision Validation</t>
         </is>
       </c>
       <c r="W90" t="inlineStr">
         <is>
-          <t>EAO-32</t>
+          <t>EAO-25</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="118" t="n">
-        <v>46266</v>
+        <v>46235</v>
       </c>
       <c r="B91" s="119" t="n">
-        <v>46267</v>
+        <v>46251</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Geopolitical</t>
+          <t>Transport Disruption</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Caterpillar</t>
+          <t>Eaton</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -12382,27 +12382,27 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Taiwan Strait Conflict Risk Assessment – Missed EventWatch Notification</t>
+          <t>Kandla Port Cargo Congestion – Supplier Impact Notification Clarification (Eaton)</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Complaint</t>
+          <t>Inquiry</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Missed Event</t>
+          <t>Supplier Impact Mapping Clarification</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>People</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Event Identification</t>
+          <t>Mapping</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -12412,66 +12412,66 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Clarification Provided</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>Geopolitical conflict risk-assessment scenario monitoring and escalation</t>
+          <t>Impact-confirmation notification criteria documentation for port/logistics bulletins</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>Staged from Jira EAO-33 (In Progress). Caterpillar reported no notification for “Taiwan Strait Conflict Risk Assessment and Potential Global Supply Chain Impact”; CS found no matching event in the backend.</t>
+          <t>Staged from Jira EAO-28 (Done). Eaton asked what criteria triggered impact-confirmation notifications to Eaton suppliers on the Kandla Port cargo congestion bulletin, since the bulletin text focused on rice exports.</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="R91" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T91" s="118" t="n">
-        <v>46266</v>
+        <v>46235</v>
       </c>
       <c r="U91" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="V91" t="inlineStr">
         <is>
-          <t>WarRoom &amp; Decision Validation</t>
+          <t>Entity &amp; Supplier Resolution</t>
         </is>
       </c>
       <c r="W91" t="inlineStr">
         <is>
-          <t>EAO-33</t>
+          <t>EAO-28</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="118" t="n">
-        <v>46266</v>
+        <v>46235</v>
       </c>
       <c r="B92" s="119" t="n">
-        <v>46268</v>
+        <v>46265</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Protest/Riot</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Ford</t>
+          <t>Liberty Blume</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -12479,27 +12479,27 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Western Balkans Truck Driver/EU Border Blockade – August 31 Update Missed Alert (Ford)</t>
+          <t>Ciena 400G Optics Counterfeit Risk Intelligence Request (Liberty Blume)</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Complaint</t>
+          <t>Inquiry</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Missed Event</t>
+          <t>Intelligence/Advisory Request</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>People</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Process Clarification</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -12514,61 +12514,61 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>Recurring/evolving-event WarRoom update monitoring and re-escalation detection</t>
+          <t>Counterfeit/grey-market component intelligence briefing capability</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>Staged from Jira EAO-34 (Open). Ford reported a missed alert for the August 31 update to Western Balkans/Serbia-EU border blockade disruptions; CS found the original January 2026 event but needs to confirm whether it was updated to cover this development. Related to the January 2026 Eaton row above (same underlying WarRoom, different customer/date).</t>
+          <t>Staged from Jira EAO-32 (Open). Liberty Blume requested industry intelligence on counterfeit/grey-market Ciena 400G optical transceivers beyond the supplier scanning report already provided.</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="R92" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T92" s="118" t="n">
-        <v>46266</v>
+        <v>46235</v>
       </c>
       <c r="U92" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="V92" t="inlineStr">
         <is>
-          <t>WarRoom &amp; Decision Validation</t>
+          <t>Other Control Automation</t>
         </is>
       </c>
       <c r="W92" t="inlineStr">
         <is>
-          <t>EAO-34</t>
+          <t>EAO-32</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="118" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="B93" s="119" t="n">
-        <v>46237</v>
+        <v>46267</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Factory Fire</t>
+          <t>Geopolitical</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>Caterpillar</t>
         </is>
       </c>
       <c r="E93" t="n">
@@ -12576,7 +12576,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Fire at UTAS-Nova Automotive Lighting Systems, Danyang, Jiangsu, China</t>
+          <t>Taiwan Strait Conflict Risk Assessment – Missed EventWatch Notification</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -12591,12 +12591,12 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>People</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Source Coverage</t>
+          <t>Event Identification</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -12611,7 +12611,7 @@
       </c>
       <c r="M93" t="inlineStr">
         <is>
-          <t>Chinese regional source coverage for sub-tier automotive lighting suppliers</t>
+          <t>Geopolitical conflict risk-assessment scenario monitoring and escalation</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -12621,7 +12621,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>Staged from Jira EAO-25 (Sent to PM). GM reported a fire at UTAS-Nova Automotive Lighting Systems, Danyang, Jiangsu, China (reported July 10) was not found in GM's org; investigation findings not yet shared, Short Term Fix Status set to Pending until CS responds.</t>
+          <t>Staged from Jira EAO-33 (In Progress). Caterpillar reported no notification for “Taiwan Strait Conflict Risk Assessment and Potential Global Supply Chain Impact”; CS found no matching event in the backend.</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
@@ -12630,10 +12630,10 @@
         </is>
       </c>
       <c r="R93" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T93" s="118" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="U93" t="inlineStr">
         <is>
@@ -12642,30 +12642,30 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>Dynamic Source Discovery</t>
+          <t>WarRoom &amp; Decision Validation</t>
         </is>
       </c>
       <c r="W93" t="inlineStr">
         <is>
-          <t>EAO-25</t>
+          <t>EAO-33</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="118" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="B94" s="119" t="n">
-        <v>46237</v>
+        <v>46268</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Tornado</t>
+          <t>Protest/Riot</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>GM</t>
+          <t>Ford</t>
         </is>
       </c>
       <c r="E94" t="n">
@@ -12673,7 +12673,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Chicago Heights, Illinois Tornado – Trialco Impact Not Identified</t>
+          <t>Western Balkans Truck Driver/EU Border Blockade – August 31 Update Missed Alert (Ford)</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -12693,7 +12693,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Event Identification</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -12708,7 +12708,7 @@
       </c>
       <c r="M94" t="inlineStr">
         <is>
-          <t>Escalation automation for localized-impact tornado/storm sub-events and named-facility (Trialco) impact confirmation</t>
+          <t>Recurring/evolving-event WarRoom update monitoring and re-escalation detection</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -12718,7 +12718,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>Staged from Jira EAO-25 (Sent to PM). GM reported no event was created specifically for the July 27 Chicago Heights, Illinois tornado (broader Illinois storm alerts existed) and asked whether Trialco was identified as impacted; investigation findings not yet shared, Short Term Fix Status set to Pending until CS responds.</t>
+          <t>Staged from Jira EAO-34 (Open). Ford reported a missed alert for the August 31 update to Western Balkans/Serbia-EU border blockade disruptions; CS found the original January 2026 event but needs to confirm whether it was updated to cover this development. Related to the January 2026 Eaton row above (same underlying WarRoom, different customer/date).</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
@@ -12727,10 +12727,10 @@
         </is>
       </c>
       <c r="R94" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T94" s="118" t="n">
-        <v>46235</v>
+        <v>46266</v>
       </c>
       <c r="U94" t="inlineStr">
         <is>
@@ -12744,7 +12744,7 @@
       </c>
       <c r="W94" t="inlineStr">
         <is>
-          <t>EAO-25</t>
+          <t>EAO-34</t>
         </is>
       </c>
     </row>

</xml_diff>